<commit_message>
CREATED plan_calculator.py : this is for calculating single action at zero plan values
</commit_message>
<xml_diff>
--- a/src/tests/env_test_configs/test_configs_matrix.xlsx
+++ b/src/tests/env_test_configs/test_configs_matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Career\00. Univesity\Masters\05. Master's thesis\PPO-project-portfolio-budgeting-AI-agent\src\tests\env_test_configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46219C76-D7D4-485E-970D-785526D0A33D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC834525-3F8E-4811-8DB5-3D95BE73DA4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="PARAM_NOTES" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CONFIGS!$A$1:$DD$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CONFIGS!$A$1:$DD$7</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="231">
   <si>
     <t>IDENTITY</t>
   </si>
@@ -407,9 +407,6 @@
   </si>
   <si>
     <t>beta</t>
-  </si>
-  <si>
-    <t>TC-1LSF-R</t>
   </si>
   <si>
     <t>TC-1LMAIF-R</t>
@@ -1272,7 +1269,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DD8"/>
+  <dimension ref="A1:DD7"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1846,7 +1843,7 @@
         <v>114</v>
       </c>
       <c r="AN3" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AO3" s="6"/>
       <c r="AP3" s="6"/>
@@ -1855,7 +1852,7 @@
         <v>114</v>
       </c>
       <c r="AS3" s="6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AT3" s="6"/>
       <c r="AU3" s="6"/>
@@ -1924,10 +1921,10 @@
       <c r="CD3" s="6"/>
       <c r="CE3" s="6"/>
       <c r="CF3" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="CG3" s="22" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="CH3" s="6"/>
       <c r="CI3" s="6"/>
@@ -2037,7 +2034,7 @@
         <v>114</v>
       </c>
       <c r="AI4" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AJ4" s="6"/>
       <c r="AK4" s="6"/>
@@ -2046,7 +2043,7 @@
         <v>114</v>
       </c>
       <c r="AN4" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AO4" s="6"/>
       <c r="AP4" s="6"/>
@@ -2055,7 +2052,7 @@
         <v>114</v>
       </c>
       <c r="AS4" s="6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AT4" s="6"/>
       <c r="AU4" s="6"/>
@@ -2064,7 +2061,7 @@
         <v>114</v>
       </c>
       <c r="AX4" s="6">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="AY4" s="6"/>
       <c r="AZ4" s="6"/>
@@ -2072,8 +2069,8 @@
       <c r="BB4" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="BC4" s="6" t="s">
-        <v>118</v>
+      <c r="BC4" s="6">
+        <v>0.2</v>
       </c>
       <c r="BD4" s="6"/>
       <c r="BE4" s="6"/>
@@ -2082,7 +2079,7 @@
         <v>114</v>
       </c>
       <c r="BH4" s="6">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BI4" s="6"/>
       <c r="BJ4" s="6"/>
@@ -2124,10 +2121,10 @@
       <c r="CD4" s="6"/>
       <c r="CE4" s="6"/>
       <c r="CF4" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="CG4" s="22" t="s">
-        <v>220</v>
+        <v>216</v>
+      </c>
+      <c r="CG4" s="6" t="s">
+        <v>221</v>
       </c>
       <c r="CH4" s="6"/>
       <c r="CI4" s="6"/>
@@ -2135,35 +2132,35 @@
       <c r="CK4" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="CL4" s="6" t="s">
-        <v>115</v>
+      <c r="CL4" s="6">
+        <v>2</v>
       </c>
       <c r="CM4" s="6"/>
       <c r="CN4" s="6"/>
       <c r="CO4" s="6"/>
       <c r="CP4" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="CQ4" s="6">
-        <v>1</v>
+        <v>216</v>
+      </c>
+      <c r="CQ4" s="22" t="s">
+        <v>230</v>
       </c>
       <c r="CR4" s="6"/>
       <c r="CS4" s="6"/>
       <c r="CT4" s="6"/>
       <c r="CU4" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="CV4" s="6">
-        <v>1</v>
+        <v>216</v>
+      </c>
+      <c r="CV4" s="6" t="s">
+        <v>223</v>
       </c>
       <c r="CW4" s="6"/>
       <c r="CX4" s="6"/>
       <c r="CY4" s="6"/>
       <c r="CZ4" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="DA4" s="6">
-        <v>0</v>
+        <v>216</v>
+      </c>
+      <c r="DA4" s="6" t="s">
+        <v>225</v>
       </c>
       <c r="DB4" s="6"/>
       <c r="DC4" s="6"/>
@@ -2171,10 +2168,10 @@
     </row>
     <row r="5" spans="1:108" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>123</v>
+        <v>227</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>123</v>
+        <v>227</v>
       </c>
       <c r="C5" s="6">
         <v>0.12</v>
@@ -2182,8 +2179,8 @@
       <c r="D5" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>115</v>
+      <c r="E5" s="6">
+        <v>1</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -2227,8 +2224,8 @@
       <c r="AC5" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="AD5" s="6">
-        <v>2</v>
+      <c r="AD5" s="6" t="s">
+        <v>118</v>
       </c>
       <c r="AE5" s="6"/>
       <c r="AF5" s="6"/>
@@ -2246,7 +2243,7 @@
         <v>114</v>
       </c>
       <c r="AN5" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
@@ -2255,7 +2252,7 @@
         <v>114</v>
       </c>
       <c r="AS5" s="6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AT5" s="6"/>
       <c r="AU5" s="6"/>
@@ -2272,8 +2269,8 @@
       <c r="BB5" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="BC5" s="6">
-        <v>0.2</v>
+      <c r="BC5" s="6" t="s">
+        <v>118</v>
       </c>
       <c r="BD5" s="6"/>
       <c r="BE5" s="6"/>
@@ -2324,10 +2321,10 @@
       <c r="CD5" s="6"/>
       <c r="CE5" s="6"/>
       <c r="CF5" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="CG5" s="6" t="s">
-        <v>222</v>
+        <v>216</v>
+      </c>
+      <c r="CG5" s="22" t="s">
+        <v>228</v>
       </c>
       <c r="CH5" s="6"/>
       <c r="CI5" s="6"/>
@@ -2342,224 +2339,224 @@
       <c r="CN5" s="6"/>
       <c r="CO5" s="6"/>
       <c r="CP5" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="CQ5" s="22" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="CR5" s="6"/>
       <c r="CS5" s="6"/>
       <c r="CT5" s="6"/>
-      <c r="CU5" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="CV5" s="6" t="s">
-        <v>224</v>
-      </c>
+      <c r="CU5" s="6"/>
+      <c r="CV5" s="6"/>
       <c r="CW5" s="6"/>
       <c r="CX5" s="6"/>
       <c r="CY5" s="6"/>
-      <c r="CZ5" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="DA5" s="6" t="s">
-        <v>226</v>
-      </c>
+      <c r="CZ5" s="6"/>
+      <c r="DA5" s="6"/>
       <c r="DB5" s="6"/>
       <c r="DC5" s="6"/>
       <c r="DD5" s="6"/>
     </row>
     <row r="6" spans="1:108" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="C6" s="6">
+      <c r="A6" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6" s="9">
         <v>0.12</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="E6" s="6">
+      <c r="D6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="J6" s="9">
+        <v>3</v>
+      </c>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="O6" s="9">
+        <v>0.95</v>
+      </c>
+      <c r="P6" s="9"/>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="T6" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="U6" s="9"/>
+      <c r="V6" s="9"/>
+      <c r="W6" s="9"/>
+      <c r="X6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y6" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="Z6" s="9"/>
+      <c r="AA6" s="9"/>
+      <c r="AB6" s="9"/>
+      <c r="AC6" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="AD6" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="AE6" s="9"/>
+      <c r="AF6" s="9"/>
+      <c r="AG6" s="9"/>
+      <c r="AH6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="AI6" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ6" s="6"/>
+      <c r="AK6" s="9"/>
+      <c r="AL6" s="9"/>
+      <c r="AM6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="AN6" s="9">
+        <v>6</v>
+      </c>
+      <c r="AO6" s="9"/>
+      <c r="AP6" s="9"/>
+      <c r="AQ6" s="9"/>
+      <c r="AR6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="AS6" s="9">
+        <v>6</v>
+      </c>
+      <c r="AT6" s="9"/>
+      <c r="AU6" s="9"/>
+      <c r="AV6" s="9"/>
+      <c r="AW6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="AX6" s="9">
+        <v>0</v>
+      </c>
+      <c r="AY6" s="9"/>
+      <c r="AZ6" s="9"/>
+      <c r="BA6" s="9"/>
+      <c r="BB6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="BC6" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="BD6" s="9"/>
+      <c r="BE6" s="9"/>
+      <c r="BF6" s="9"/>
+      <c r="BG6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="BH6" s="9">
+        <v>0</v>
+      </c>
+      <c r="BI6" s="9"/>
+      <c r="BJ6" s="9"/>
+      <c r="BK6" s="9"/>
+      <c r="BL6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="BM6" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="BN6" s="9"/>
+      <c r="BO6" s="9"/>
+      <c r="BP6" s="9"/>
+      <c r="BQ6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="BR6" s="9">
+        <v>0.15</v>
+      </c>
+      <c r="BS6" s="9"/>
+      <c r="BT6" s="9"/>
+      <c r="BU6" s="9"/>
+      <c r="BV6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="BW6" s="9">
+        <v>2</v>
+      </c>
+      <c r="BX6" s="9"/>
+      <c r="BY6" s="9"/>
+      <c r="BZ6" s="9"/>
+      <c r="CA6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="CB6" s="9">
+        <v>2</v>
+      </c>
+      <c r="CC6" s="9"/>
+      <c r="CD6" s="9"/>
+      <c r="CE6" s="9"/>
+      <c r="CF6" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="CG6" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="CH6" s="9"/>
+      <c r="CI6" s="9"/>
+      <c r="CJ6" s="9"/>
+      <c r="CK6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="CL6" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="CM6" s="9"/>
+      <c r="CN6" s="9"/>
+      <c r="CO6" s="9"/>
+      <c r="CP6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="CQ6" s="9">
         <v>1</v>
       </c>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="J6" s="6">
-        <v>3</v>
-      </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="O6" s="6">
-        <v>0.95</v>
-      </c>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="T6" s="6">
-        <v>100</v>
-      </c>
-      <c r="U6" s="6"/>
-      <c r="V6" s="6"/>
-      <c r="W6" s="6"/>
-      <c r="X6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y6" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="Z6" s="6"/>
-      <c r="AA6" s="6"/>
-      <c r="AB6" s="6"/>
-      <c r="AC6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="AD6" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="AE6" s="6"/>
-      <c r="AF6" s="6"/>
-      <c r="AG6" s="6"/>
-      <c r="AH6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="AI6" s="6">
-        <v>3</v>
-      </c>
-      <c r="AJ6" s="6"/>
-      <c r="AK6" s="6"/>
-      <c r="AL6" s="6"/>
-      <c r="AM6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="AN6" s="6">
-        <v>2</v>
-      </c>
-      <c r="AO6" s="6"/>
-      <c r="AP6" s="6"/>
-      <c r="AQ6" s="6"/>
-      <c r="AR6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="AS6" s="6">
-        <v>5</v>
-      </c>
-      <c r="AT6" s="6"/>
-      <c r="AU6" s="6"/>
-      <c r="AV6" s="6"/>
-      <c r="AW6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="AX6" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="AY6" s="6"/>
-      <c r="AZ6" s="6"/>
-      <c r="BA6" s="6"/>
-      <c r="BB6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="BC6" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="BD6" s="6"/>
-      <c r="BE6" s="6"/>
-      <c r="BF6" s="6"/>
-      <c r="BG6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="BH6" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="BI6" s="6"/>
-      <c r="BJ6" s="6"/>
-      <c r="BK6" s="6"/>
-      <c r="BL6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="BM6" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="BN6" s="6"/>
-      <c r="BO6" s="6"/>
-      <c r="BP6" s="6"/>
-      <c r="BQ6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="BR6" s="6">
-        <v>0.15</v>
-      </c>
-      <c r="BS6" s="6"/>
-      <c r="BT6" s="6"/>
-      <c r="BU6" s="6"/>
-      <c r="BV6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="BW6" s="6">
-        <v>2</v>
-      </c>
-      <c r="BX6" s="6"/>
-      <c r="BY6" s="6"/>
-      <c r="BZ6" s="6"/>
-      <c r="CA6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="CB6" s="6">
-        <v>2</v>
-      </c>
-      <c r="CC6" s="6"/>
-      <c r="CD6" s="6"/>
-      <c r="CE6" s="6"/>
-      <c r="CF6" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="CG6" s="22" t="s">
-        <v>229</v>
-      </c>
-      <c r="CH6" s="6"/>
-      <c r="CI6" s="6"/>
-      <c r="CJ6" s="6"/>
-      <c r="CK6" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="CL6" s="6">
-        <v>2</v>
-      </c>
-      <c r="CM6" s="6"/>
-      <c r="CN6" s="6"/>
-      <c r="CO6" s="6"/>
-      <c r="CP6" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="CQ6" s="22" t="s">
-        <v>230</v>
-      </c>
-      <c r="CR6" s="6"/>
-      <c r="CS6" s="6"/>
-      <c r="CT6" s="6"/>
-      <c r="CU6" s="6"/>
-      <c r="CV6" s="6"/>
-      <c r="CW6" s="6"/>
-      <c r="CX6" s="6"/>
-      <c r="CY6" s="6"/>
-      <c r="CZ6" s="6"/>
-      <c r="DA6" s="6"/>
-      <c r="DB6" s="6"/>
-      <c r="DC6" s="6"/>
-      <c r="DD6" s="6"/>
+      <c r="CR6" s="9"/>
+      <c r="CS6" s="9"/>
+      <c r="CT6" s="9"/>
+      <c r="CU6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="CV6" s="9">
+        <v>1</v>
+      </c>
+      <c r="CW6" s="9"/>
+      <c r="CX6" s="9"/>
+      <c r="CY6" s="9"/>
+      <c r="CZ6" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="DA6" s="9">
+        <v>0</v>
+      </c>
+      <c r="DB6" s="9"/>
+      <c r="DC6" s="9"/>
+      <c r="DD6" s="9"/>
     </row>
     <row r="7" spans="1:108" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
@@ -2599,10 +2596,10 @@
       <c r="Q7" s="9"/>
       <c r="R7" s="9"/>
       <c r="S7" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="T7" s="9" t="s">
         <v>217</v>
-      </c>
-      <c r="T7" s="9" t="s">
-        <v>218</v>
       </c>
       <c r="U7" s="9"/>
       <c r="V7" s="9"/>
@@ -2617,10 +2614,10 @@
       <c r="AA7" s="9"/>
       <c r="AB7" s="9"/>
       <c r="AC7" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AD7" s="9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AE7" s="9"/>
       <c r="AF7" s="9"/>
@@ -2629,7 +2626,7 @@
         <v>114</v>
       </c>
       <c r="AI7" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AJ7" s="6"/>
       <c r="AK7" s="9"/>
@@ -2638,7 +2635,7 @@
         <v>114</v>
       </c>
       <c r="AN7" s="9">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AO7" s="9"/>
       <c r="AP7" s="9"/>
@@ -2647,7 +2644,7 @@
         <v>114</v>
       </c>
       <c r="AS7" s="9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AT7" s="9"/>
       <c r="AU7" s="9"/>
@@ -2656,7 +2653,7 @@
         <v>114</v>
       </c>
       <c r="AX7" s="9">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="AY7" s="9"/>
       <c r="AZ7" s="9"/>
@@ -2674,7 +2671,7 @@
         <v>114</v>
       </c>
       <c r="BH7" s="9">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BI7" s="9"/>
       <c r="BJ7" s="9"/>
@@ -2716,10 +2713,10 @@
       <c r="CD7" s="9"/>
       <c r="CE7" s="9"/>
       <c r="CF7" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="CG7" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="CH7" s="9"/>
       <c r="CI7" s="9"/>
@@ -2727,242 +2724,42 @@
       <c r="CK7" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="CL7" s="9" t="s">
-        <v>115</v>
+      <c r="CL7" s="9">
+        <v>3</v>
       </c>
       <c r="CM7" s="9"/>
       <c r="CN7" s="9"/>
       <c r="CO7" s="9"/>
       <c r="CP7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="CQ7" s="9">
-        <v>1</v>
+        <v>216</v>
+      </c>
+      <c r="CQ7" s="9" t="s">
+        <v>224</v>
       </c>
       <c r="CR7" s="9"/>
       <c r="CS7" s="9"/>
       <c r="CT7" s="9"/>
       <c r="CU7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="CV7" s="9">
-        <v>1</v>
+        <v>216</v>
+      </c>
+      <c r="CV7" s="9" t="s">
+        <v>224</v>
       </c>
       <c r="CW7" s="9"/>
       <c r="CX7" s="9"/>
       <c r="CY7" s="9"/>
       <c r="CZ7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="DA7" s="9">
-        <v>0</v>
+        <v>216</v>
+      </c>
+      <c r="DA7" s="9" t="s">
+        <v>226</v>
       </c>
       <c r="DB7" s="9"/>
       <c r="DC7" s="9"/>
       <c r="DD7" s="9"/>
     </row>
-    <row r="8" spans="1:108" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="C8" s="9">
-        <v>0.12</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="J8" s="9">
-        <v>3</v>
-      </c>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="O8" s="9">
-        <v>0.95</v>
-      </c>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="9"/>
-      <c r="S8" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="T8" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
-      <c r="W8" s="9"/>
-      <c r="X8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y8" s="9">
-        <v>0.2</v>
-      </c>
-      <c r="Z8" s="9"/>
-      <c r="AA8" s="9"/>
-      <c r="AB8" s="9"/>
-      <c r="AC8" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="AD8" s="9" t="s">
-        <v>219</v>
-      </c>
-      <c r="AE8" s="9"/>
-      <c r="AF8" s="9"/>
-      <c r="AG8" s="9"/>
-      <c r="AH8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AI8" s="9">
-        <v>3</v>
-      </c>
-      <c r="AJ8" s="6"/>
-      <c r="AK8" s="9"/>
-      <c r="AL8" s="9"/>
-      <c r="AM8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AN8" s="9">
-        <v>2</v>
-      </c>
-      <c r="AO8" s="9"/>
-      <c r="AP8" s="9"/>
-      <c r="AQ8" s="9"/>
-      <c r="AR8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AS8" s="9">
-        <v>5</v>
-      </c>
-      <c r="AT8" s="9"/>
-      <c r="AU8" s="9"/>
-      <c r="AV8" s="9"/>
-      <c r="AW8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AX8" s="9">
-        <v>0.2</v>
-      </c>
-      <c r="AY8" s="9"/>
-      <c r="AZ8" s="9"/>
-      <c r="BA8" s="9"/>
-      <c r="BB8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="BC8" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="BD8" s="9"/>
-      <c r="BE8" s="9"/>
-      <c r="BF8" s="9"/>
-      <c r="BG8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="BH8" s="9">
-        <v>0.2</v>
-      </c>
-      <c r="BI8" s="9"/>
-      <c r="BJ8" s="9"/>
-      <c r="BK8" s="9"/>
-      <c r="BL8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="BM8" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="BN8" s="9"/>
-      <c r="BO8" s="9"/>
-      <c r="BP8" s="9"/>
-      <c r="BQ8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="BR8" s="9">
-        <v>0.15</v>
-      </c>
-      <c r="BS8" s="9"/>
-      <c r="BT8" s="9"/>
-      <c r="BU8" s="9"/>
-      <c r="BV8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="BW8" s="9">
-        <v>2</v>
-      </c>
-      <c r="BX8" s="9"/>
-      <c r="BY8" s="9"/>
-      <c r="BZ8" s="9"/>
-      <c r="CA8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="CB8" s="9">
-        <v>2</v>
-      </c>
-      <c r="CC8" s="9"/>
-      <c r="CD8" s="9"/>
-      <c r="CE8" s="9"/>
-      <c r="CF8" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="CG8" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="CH8" s="9"/>
-      <c r="CI8" s="9"/>
-      <c r="CJ8" s="9"/>
-      <c r="CK8" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="CL8" s="9">
-        <v>3</v>
-      </c>
-      <c r="CM8" s="9"/>
-      <c r="CN8" s="9"/>
-      <c r="CO8" s="9"/>
-      <c r="CP8" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="CQ8" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="CR8" s="9"/>
-      <c r="CS8" s="9"/>
-      <c r="CT8" s="9"/>
-      <c r="CU8" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="CV8" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="CW8" s="9"/>
-      <c r="CX8" s="9"/>
-      <c r="CY8" s="9"/>
-      <c r="CZ8" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="DA8" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="DB8" s="9"/>
-      <c r="DC8" s="9"/>
-      <c r="DD8" s="9"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:DD8" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:DD7" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="3" showButton="0"/>
     <filterColumn colId="4" showButton="0"/>
     <filterColumn colId="5" showButton="0"/>
@@ -3073,7 +2870,7 @@
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid distribution" error="Choose from the dropdown list." sqref="S9:S18 CK3:CK18 AC3:AC18 CA3:CA18 BV3:BV18 BQ3:BQ18 BL3:BL18 BG3:BG18 BB3:BB18 AW3:AW18 AR3:AR18 AM3:AM18 I3:I18 AH3:AH18 X3:X18 D3:D18 N3:N18 CZ3:CZ18 CF3:CF18 CU3:CU18 CP3:CP18" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid distribution" error="Choose from the dropdown list." sqref="S8:S17 CP3:CP17 CU3:CU17 CF3:CF17 CZ3:CZ17 N3:N17 D3:D17 X3:X17 AH3:AH17 I3:I17 AM3:AM17 AR3:AR17 AW3:AW17 BB3:BB17 BG3:BG17 BL3:BL17 BQ3:BQ17 BV3:BV17 CA3:CA17 AC3:AC17 CK3:CK17" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"fixed,uniform,triangular,normal,lognormal,beta,poisson,discrete"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3098,7 +2895,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -3109,154 +2906,154 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>127</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>128</v>
       </c>
       <c r="C3" s="10"/>
       <c r="D3" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="D4" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>135</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>137</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>138</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>117</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="D6" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="E6" s="12" t="s">
         <v>142</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="D7" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="E7" s="12" t="s">
         <v>146</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>148</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>149</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>116</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>151</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>152</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>121</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="B10" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="D10" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="E10" s="12" t="s">
         <v>156</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="D11" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="E11" s="12" t="s">
         <v>160</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="B12" s="12" t="s">
         <v>162</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>164</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -3281,7 +3078,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -3289,21 +3086,21 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="D2" s="10" t="s">
         <v>169</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>2</v>
@@ -3312,12 +3109,12 @@
         <v>114</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>2</v>
@@ -3326,12 +3123,12 @@
         <v>116</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="14" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>2</v>
@@ -3340,12 +3137,12 @@
         <v>117</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>2</v>
@@ -3354,12 +3151,12 @@
         <v>114</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B7" s="18" t="s">
         <v>3</v>
@@ -3368,12 +3165,12 @@
         <v>116</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="17" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B8" s="18" t="s">
         <v>3</v>
@@ -3382,12 +3179,12 @@
         <v>117</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B9" s="18" t="s">
         <v>3</v>
@@ -3396,12 +3193,12 @@
         <v>114</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B10" s="18" t="s">
         <v>3</v>
@@ -3410,12 +3207,12 @@
         <v>117</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B11" s="18" t="s">
         <v>3</v>
@@ -3424,12 +3221,12 @@
         <v>117</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="17" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B12" s="18" t="s">
         <v>3</v>
@@ -3438,12 +3235,12 @@
         <v>117</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B13" s="18" t="s">
         <v>3</v>
@@ -3452,12 +3249,12 @@
         <v>117</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="17" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B14" s="18" t="s">
         <v>3</v>
@@ -3466,12 +3263,12 @@
         <v>114</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="17" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B15" s="18" t="s">
         <v>3</v>
@@ -3480,12 +3277,12 @@
         <v>117</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="17" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B16" s="18" t="s">
         <v>3</v>
@@ -3494,12 +3291,12 @@
         <v>117</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B17" s="18" t="s">
         <v>3</v>
@@ -3508,12 +3305,12 @@
         <v>117</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B18" s="18" t="s">
         <v>3</v>
@@ -3522,12 +3319,12 @@
         <v>117</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B19" s="18" t="s">
         <v>3</v>
@@ -3536,12 +3333,12 @@
         <v>117</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="17" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B20" s="18" t="s">
         <v>3</v>
@@ -3550,12 +3347,12 @@
         <v>117</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B21" s="18" t="s">
         <v>3</v>
@@ -3564,12 +3361,12 @@
         <v>114</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B22" s="8" t="s">
         <v>4</v>
@@ -3578,12 +3375,12 @@
         <v>114</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>4</v>
@@ -3592,12 +3389,12 @@
         <v>117</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="20" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B24" s="8" t="s">
         <v>4</v>
@@ -3606,12 +3403,12 @@
         <v>117</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>4</v>
@@ -3620,7 +3417,7 @@
         <v>117</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATED tests\* : updated the matrix to include all the cases and scenarios
</commit_message>
<xml_diff>
--- a/src/tests/env_test_configs/test_configs_matrix.xlsx
+++ b/src/tests/env_test_configs/test_configs_matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Career\00. Univesity\Masters\05. Master's thesis\PPO-project-portfolio-budgeting-AI-agent\src\tests\env_test_configs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\0. Univesity\Masters\05. Master's thesis\PPO-project-portfolio-budgeting-AI-agent\src\tests\env_test_configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC834525-3F8E-4811-8DB5-3D95BE73DA4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDA92E8D-6127-42B3-B3E0-3D5452556639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="PARAM_NOTES" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CONFIGS!$A$1:$DD$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CONFIGS!$A$1:$DD$6</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="229">
   <si>
     <t>IDENTITY</t>
   </si>
@@ -412,9 +412,6 @@
     <t>TC-1LMAIF-R</t>
   </si>
   <si>
-    <t>TC-3XSF-R</t>
-  </si>
-  <si>
     <t>TC-3XMAIF-R</t>
   </si>
   <si>
@@ -697,27 +694,15 @@
     <t>[100, 200, 300]</t>
   </si>
   <si>
-    <t>[0, 2, 4]</t>
-  </si>
-  <si>
     <t>[0.91, 1.17, 0.83]</t>
   </si>
   <si>
-    <t>[[0.91, 1.17, 0.83],[1.09, 0.84, 1.18],[0.97,1.13,0.86]]</t>
-  </si>
-  <si>
     <t>[0.91, 1.17, 0.83, 0.91, 1.17, 0.83]</t>
   </si>
   <si>
     <t>[[0.91, 1.17, 0.83 ,0.91, 1.17, 0.83],[1.09, 0.84, 1.18 ,1.09, 0.84, 1.18],[0.97,1.13,0.86 ,0.97,1.13,0.86]]</t>
   </si>
   <si>
-    <t>[0.3, 0.6, 1.0]</t>
-  </si>
-  <si>
-    <t>[[0.3, 0.6, 1.0],[0.3, 0.6, 1.0],[0.3, 0.6, 1.0]]</t>
-  </si>
-  <si>
     <t>[1, 2, 3]</t>
   </si>
   <si>
@@ -727,13 +712,22 @@
     <t>TC-10MAIF-R</t>
   </si>
   <si>
-    <t>[0.91, 0.83, 0.87, 0.65, 0.50, 0.72]</t>
-  </si>
-  <si>
-    <t>[0.3, 1.0]</t>
-  </si>
-  <si>
-    <t>[0.1, 1.0]</t>
+    <t>[0.4, 0.97, 1.0]</t>
+  </si>
+  <si>
+    <t>[0.3, 0.7, 1.0]</t>
+  </si>
+  <si>
+    <t>[[0.4, 0.97, 1.0],[0.4, 0.97, 1.0],[0.4, 0.97, 1.0]]</t>
+  </si>
+  <si>
+    <t>[[0.3, 0.7, 1.0],[0.3, 0.7, 1.0],[0.3, 0.7, 1.0]]</t>
+  </si>
+  <si>
+    <t>[0.95, 0.91, 0.55, 0.40, 0.30, 0.20]</t>
+  </si>
+  <si>
+    <t>[0, 6, 7]</t>
   </si>
 </sst>
 </file>
@@ -1269,7 +1263,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DD7"/>
+  <dimension ref="A1:DD6"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1843,7 +1837,7 @@
         <v>114</v>
       </c>
       <c r="AN3" s="6">
-        <v>6</v>
+        <v>1.5</v>
       </c>
       <c r="AO3" s="6"/>
       <c r="AP3" s="6"/>
@@ -1852,7 +1846,7 @@
         <v>114</v>
       </c>
       <c r="AS3" s="6">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AT3" s="6"/>
       <c r="AU3" s="6"/>
@@ -1921,10 +1915,10 @@
       <c r="CD3" s="6"/>
       <c r="CE3" s="6"/>
       <c r="CF3" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="CG3" s="22" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="CH3" s="6"/>
       <c r="CI3" s="6"/>
@@ -2043,7 +2037,7 @@
         <v>114</v>
       </c>
       <c r="AN4" s="6">
-        <v>6</v>
+        <v>1.5</v>
       </c>
       <c r="AO4" s="6"/>
       <c r="AP4" s="6"/>
@@ -2052,7 +2046,7 @@
         <v>114</v>
       </c>
       <c r="AS4" s="6">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AT4" s="6"/>
       <c r="AU4" s="6"/>
@@ -2070,7 +2064,7 @@
         <v>114</v>
       </c>
       <c r="BC4" s="6">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="BD4" s="6"/>
       <c r="BE4" s="6"/>
@@ -2079,7 +2073,7 @@
         <v>114</v>
       </c>
       <c r="BH4" s="6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="BI4" s="6"/>
       <c r="BJ4" s="6"/>
@@ -2121,10 +2115,10 @@
       <c r="CD4" s="6"/>
       <c r="CE4" s="6"/>
       <c r="CF4" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="CG4" s="6" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="CH4" s="6"/>
       <c r="CI4" s="6"/>
@@ -2133,34 +2127,34 @@
         <v>114</v>
       </c>
       <c r="CL4" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CM4" s="6"/>
       <c r="CN4" s="6"/>
       <c r="CO4" s="6"/>
       <c r="CP4" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="CQ4" s="22" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="CR4" s="6"/>
       <c r="CS4" s="6"/>
       <c r="CT4" s="6"/>
       <c r="CU4" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="CV4" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="CW4" s="6"/>
       <c r="CX4" s="6"/>
       <c r="CY4" s="6"/>
       <c r="CZ4" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="DA4" s="6" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="DB4" s="6"/>
       <c r="DC4" s="6"/>
@@ -2168,10 +2162,10 @@
     </row>
     <row r="5" spans="1:108" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="C5" s="6">
         <v>0.12</v>
@@ -2243,7 +2237,7 @@
         <v>114</v>
       </c>
       <c r="AN5" s="6">
-        <v>6</v>
+        <v>1.5</v>
       </c>
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
@@ -2252,7 +2246,7 @@
         <v>114</v>
       </c>
       <c r="AS5" s="6">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AT5" s="6"/>
       <c r="AU5" s="6"/>
@@ -2321,10 +2315,10 @@
       <c r="CD5" s="6"/>
       <c r="CE5" s="6"/>
       <c r="CF5" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="CG5" s="22" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="CH5" s="6"/>
       <c r="CI5" s="6"/>
@@ -2333,27 +2327,35 @@
         <v>114</v>
       </c>
       <c r="CL5" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CM5" s="6"/>
       <c r="CN5" s="6"/>
       <c r="CO5" s="6"/>
       <c r="CP5" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="CQ5" s="22" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="CR5" s="6"/>
       <c r="CS5" s="6"/>
       <c r="CT5" s="6"/>
-      <c r="CU5" s="6"/>
-      <c r="CV5" s="6"/>
+      <c r="CU5" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="CV5" s="6" t="s">
+        <v>224</v>
+      </c>
       <c r="CW5" s="6"/>
       <c r="CX5" s="6"/>
       <c r="CY5" s="6"/>
-      <c r="CZ5" s="6"/>
-      <c r="DA5" s="6"/>
+      <c r="CZ5" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="DA5" s="6" t="s">
+        <v>220</v>
+      </c>
       <c r="DB5" s="6"/>
       <c r="DC5" s="6"/>
       <c r="DD5" s="6"/>
@@ -2396,10 +2398,10 @@
       <c r="Q6" s="9"/>
       <c r="R6" s="9"/>
       <c r="S6" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="T6" s="9" t="s">
         <v>216</v>
-      </c>
-      <c r="T6" s="9" t="s">
-        <v>217</v>
       </c>
       <c r="U6" s="9"/>
       <c r="V6" s="9"/>
@@ -2414,10 +2416,10 @@
       <c r="AA6" s="9"/>
       <c r="AB6" s="9"/>
       <c r="AC6" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="AD6" s="9" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="AE6" s="9"/>
       <c r="AF6" s="9"/>
@@ -2426,16 +2428,16 @@
         <v>114</v>
       </c>
       <c r="AI6" s="9">
-        <v>0</v>
-      </c>
-      <c r="AJ6" s="6"/>
+        <v>3</v>
+      </c>
+      <c r="AJ6" s="9"/>
       <c r="AK6" s="9"/>
       <c r="AL6" s="9"/>
       <c r="AM6" s="9" t="s">
         <v>114</v>
       </c>
       <c r="AN6" s="9">
-        <v>6</v>
+        <v>1.5</v>
       </c>
       <c r="AO6" s="9"/>
       <c r="AP6" s="9"/>
@@ -2444,7 +2446,7 @@
         <v>114</v>
       </c>
       <c r="AS6" s="9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AT6" s="9"/>
       <c r="AU6" s="9"/>
@@ -2453,7 +2455,7 @@
         <v>114</v>
       </c>
       <c r="AX6" s="9">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="AY6" s="9"/>
       <c r="AZ6" s="9"/>
@@ -2471,7 +2473,7 @@
         <v>114</v>
       </c>
       <c r="BH6" s="9">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BI6" s="9"/>
       <c r="BJ6" s="9"/>
@@ -2513,10 +2515,10 @@
       <c r="CD6" s="9"/>
       <c r="CE6" s="9"/>
       <c r="CF6" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="CG6" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="CH6" s="9"/>
       <c r="CI6" s="9"/>
@@ -2524,242 +2526,42 @@
       <c r="CK6" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="CL6" s="9" t="s">
-        <v>115</v>
+      <c r="CL6" s="9">
+        <v>3</v>
       </c>
       <c r="CM6" s="9"/>
       <c r="CN6" s="9"/>
       <c r="CO6" s="9"/>
       <c r="CP6" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="CQ6" s="9">
-        <v>1</v>
+        <v>215</v>
+      </c>
+      <c r="CQ6" s="9" t="s">
+        <v>225</v>
       </c>
       <c r="CR6" s="9"/>
       <c r="CS6" s="9"/>
       <c r="CT6" s="9"/>
       <c r="CU6" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="CV6" s="9">
-        <v>1</v>
+        <v>215</v>
+      </c>
+      <c r="CV6" s="9" t="s">
+        <v>226</v>
       </c>
       <c r="CW6" s="9"/>
       <c r="CX6" s="9"/>
       <c r="CY6" s="9"/>
       <c r="CZ6" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="DA6" s="9">
-        <v>0</v>
+        <v>215</v>
+      </c>
+      <c r="DA6" s="9" t="s">
+        <v>221</v>
       </c>
       <c r="DB6" s="9"/>
       <c r="DC6" s="9"/>
       <c r="DD6" s="9"/>
     </row>
-    <row r="7" spans="1:108" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="C7" s="9">
-        <v>0.12</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="J7" s="9">
-        <v>3</v>
-      </c>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="O7" s="9">
-        <v>0.95</v>
-      </c>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="9"/>
-      <c r="S7" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="T7" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9"/>
-      <c r="W7" s="9"/>
-      <c r="X7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y7" s="9">
-        <v>0.2</v>
-      </c>
-      <c r="Z7" s="9"/>
-      <c r="AA7" s="9"/>
-      <c r="AB7" s="9"/>
-      <c r="AC7" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="AD7" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="AE7" s="9"/>
-      <c r="AF7" s="9"/>
-      <c r="AG7" s="9"/>
-      <c r="AH7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AI7" s="9">
-        <v>3</v>
-      </c>
-      <c r="AJ7" s="6"/>
-      <c r="AK7" s="9"/>
-      <c r="AL7" s="9"/>
-      <c r="AM7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AN7" s="9">
-        <v>6</v>
-      </c>
-      <c r="AO7" s="9"/>
-      <c r="AP7" s="9"/>
-      <c r="AQ7" s="9"/>
-      <c r="AR7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AS7" s="9">
-        <v>6</v>
-      </c>
-      <c r="AT7" s="9"/>
-      <c r="AU7" s="9"/>
-      <c r="AV7" s="9"/>
-      <c r="AW7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AX7" s="9">
-        <v>0.2</v>
-      </c>
-      <c r="AY7" s="9"/>
-      <c r="AZ7" s="9"/>
-      <c r="BA7" s="9"/>
-      <c r="BB7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="BC7" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="BD7" s="9"/>
-      <c r="BE7" s="9"/>
-      <c r="BF7" s="9"/>
-      <c r="BG7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="BH7" s="9">
-        <v>0.2</v>
-      </c>
-      <c r="BI7" s="9"/>
-      <c r="BJ7" s="9"/>
-      <c r="BK7" s="9"/>
-      <c r="BL7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="BM7" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="BN7" s="9"/>
-      <c r="BO7" s="9"/>
-      <c r="BP7" s="9"/>
-      <c r="BQ7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="BR7" s="9">
-        <v>0.15</v>
-      </c>
-      <c r="BS7" s="9"/>
-      <c r="BT7" s="9"/>
-      <c r="BU7" s="9"/>
-      <c r="BV7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="BW7" s="9">
-        <v>2</v>
-      </c>
-      <c r="BX7" s="9"/>
-      <c r="BY7" s="9"/>
-      <c r="BZ7" s="9"/>
-      <c r="CA7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="CB7" s="9">
-        <v>2</v>
-      </c>
-      <c r="CC7" s="9"/>
-      <c r="CD7" s="9"/>
-      <c r="CE7" s="9"/>
-      <c r="CF7" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="CG7" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="CH7" s="9"/>
-      <c r="CI7" s="9"/>
-      <c r="CJ7" s="9"/>
-      <c r="CK7" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="CL7" s="9">
-        <v>3</v>
-      </c>
-      <c r="CM7" s="9"/>
-      <c r="CN7" s="9"/>
-      <c r="CO7" s="9"/>
-      <c r="CP7" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="CQ7" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="CR7" s="9"/>
-      <c r="CS7" s="9"/>
-      <c r="CT7" s="9"/>
-      <c r="CU7" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="CV7" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="CW7" s="9"/>
-      <c r="CX7" s="9"/>
-      <c r="CY7" s="9"/>
-      <c r="CZ7" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="DA7" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="DB7" s="9"/>
-      <c r="DC7" s="9"/>
-      <c r="DD7" s="9"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:DD7" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:DD6" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="3" showButton="0"/>
     <filterColumn colId="4" showButton="0"/>
     <filterColumn colId="5" showButton="0"/>
@@ -2870,7 +2672,7 @@
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid distribution" error="Choose from the dropdown list." sqref="S8:S17 CP3:CP17 CU3:CU17 CF3:CF17 CZ3:CZ17 N3:N17 D3:D17 X3:X17 AH3:AH17 I3:I17 AM3:AM17 AR3:AR17 AW3:AW17 BB3:BB17 BG3:BG17 BL3:BL17 BQ3:BQ17 BV3:BV17 CA3:CA17 AC3:AC17 CK3:CK17" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid distribution" error="Choose from the dropdown list." sqref="S7:S16 CZ3:CZ16 AC3:AC16 CA3:CA16 BV3:BV16 BQ3:BQ16 BL3:BL16 BG3:BG16 BB3:BB16 AW3:AW16 AR3:AR16 AM3:AM16 I3:I16 AH3:AH16 X3:X16 D3:D16 N3:N16 CU3:CU16 CF3:CF16 CK3:CK16 CP3:CP16" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"fixed,uniform,triangular,normal,lognormal,beta,poisson,discrete"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2895,7 +2697,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -2906,154 +2708,154 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>126</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>127</v>
       </c>
       <c r="C3" s="10"/>
       <c r="D3" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>131</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="D4" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>134</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>136</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>137</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>117</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="D6" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="E6" s="12" t="s">
         <v>141</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="D7" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="E7" s="12" t="s">
         <v>145</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>147</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>148</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>116</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>150</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>151</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>121</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="B10" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="D10" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="E10" s="12" t="s">
         <v>155</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="D11" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="E11" s="12" t="s">
         <v>159</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="B12" s="12" t="s">
         <v>161</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -3078,7 +2880,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -3086,21 +2888,21 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="D2" s="10" t="s">
         <v>168</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>2</v>
@@ -3109,12 +2911,12 @@
         <v>114</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>2</v>
@@ -3123,12 +2925,12 @@
         <v>116</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>2</v>
@@ -3137,12 +2939,12 @@
         <v>117</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>2</v>
@@ -3151,12 +2953,12 @@
         <v>114</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B7" s="18" t="s">
         <v>3</v>
@@ -3165,12 +2967,12 @@
         <v>116</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B8" s="18" t="s">
         <v>3</v>
@@ -3179,12 +2981,12 @@
         <v>117</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B9" s="18" t="s">
         <v>3</v>
@@ -3193,12 +2995,12 @@
         <v>114</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B10" s="18" t="s">
         <v>3</v>
@@ -3207,12 +3009,12 @@
         <v>117</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B11" s="18" t="s">
         <v>3</v>
@@ -3221,12 +3023,12 @@
         <v>117</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="17" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B12" s="18" t="s">
         <v>3</v>
@@ -3235,12 +3037,12 @@
         <v>117</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B13" s="18" t="s">
         <v>3</v>
@@ -3249,12 +3051,12 @@
         <v>117</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="17" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B14" s="18" t="s">
         <v>3</v>
@@ -3263,12 +3065,12 @@
         <v>114</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B15" s="18" t="s">
         <v>3</v>
@@ -3277,12 +3079,12 @@
         <v>117</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="17" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B16" s="18" t="s">
         <v>3</v>
@@ -3291,12 +3093,12 @@
         <v>117</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B17" s="18" t="s">
         <v>3</v>
@@ -3305,12 +3107,12 @@
         <v>117</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B18" s="18" t="s">
         <v>3</v>
@@ -3319,12 +3121,12 @@
         <v>117</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="17" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B19" s="18" t="s">
         <v>3</v>
@@ -3333,12 +3135,12 @@
         <v>117</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B20" s="18" t="s">
         <v>3</v>
@@ -3347,12 +3149,12 @@
         <v>117</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="17" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B21" s="18" t="s">
         <v>3</v>
@@ -3361,12 +3163,12 @@
         <v>114</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="20" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B22" s="8" t="s">
         <v>4</v>
@@ -3375,12 +3177,12 @@
         <v>114</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="20" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>4</v>
@@ -3389,12 +3191,12 @@
         <v>117</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B24" s="8" t="s">
         <v>4</v>
@@ -3403,12 +3205,12 @@
         <v>117</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>4</v>
@@ -3417,7 +3219,7 @@
         <v>117</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>